<commit_message>
Smart-Connect Board BOM with Price added.
</commit_message>
<xml_diff>
--- a/Design-Files/BB_Production/BOM/BOM-With-Price_BB_Production.xlsx
+++ b/Design-Files/BB_Production/BOM/BOM-With-Price_BB_Production.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="367" uniqueCount="209">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="364" uniqueCount="231">
   <si>
     <t>#</t>
   </si>
@@ -646,6 +646,72 @@
   </si>
   <si>
     <t>Mouser</t>
+  </si>
+  <si>
+    <t>https://lcsc.com/product-detail/multilayer-ceramic-capacitors-mlcc-smd-smt_murata-grm31cr61e476me44l_C403725.html</t>
+  </si>
+  <si>
+    <t>https://lcsc.com/product-detail/multilayer-ceramic-capacitors-mlcc-smd-smt_murata-grm155r71e104ke14d_C77014.html</t>
+  </si>
+  <si>
+    <t>https://lcsc.com/product-detail/multilayer-ceramic-capacitors-mlcc-smd-smt_yageo-cc0402jrx7r7bb104_C541464.html</t>
+  </si>
+  <si>
+    <t>https://lcsc.com/product-detail/schottky-diodes_juxing-ss510b_C3011128.html</t>
+  </si>
+  <si>
+    <t>https://lcsc.com/product-detail/esd-and-surge-protection-tvs-esd_tech-public-sm712_C521963.html</t>
+  </si>
+  <si>
+    <t>https://lcsc.com/product-detail/wire-to-board-connector_hctl-hc-1-25-16plt_C3012301.html</t>
+  </si>
+  <si>
+    <t>https://lcsc.com/product-detail/pin-headers_xkb-connection-x6511wv-02h-c60d30_C706874.html</t>
+  </si>
+  <si>
+    <t>https://lcsc.com/product-detail/inductors-smd_koherelec-mda1040-470m_C2847557.html</t>
+  </si>
+  <si>
+    <t>https://lcsc.com/product-detail/mosfets_willsemi-wnm2016a-3-tr_C601105.html</t>
+  </si>
+  <si>
+    <t>https://lcsc.com/product-detail/chip-resistor-surface-mount_yageo-rc0603jr-070rl_C95177.html</t>
+  </si>
+  <si>
+    <t>https://lcsc.com/product-detail/chip-resistor-surface-mount_yageo-rc1206jr-070rl_C108081.html</t>
+  </si>
+  <si>
+    <t>https://lcsc.com/product-detail/chip-resistor-surface-mount_yageo-rc0402fr-0710kl_C60490.html</t>
+  </si>
+  <si>
+    <t>https://lcsc.com/product-detail/chip-resistor-surface-mount_yageo-rc0402fr-070rl_C106231.html</t>
+  </si>
+  <si>
+    <t>https://lcsc.com/product-detail/chip-resistor-surface-mount_yageo-rc0603fr-07120rl_C114640.html</t>
+  </si>
+  <si>
+    <t>https://lcsc.com/product-detail/chip-resistor-surface-mount_vishay-rca0603100rfkeahp_C2074203.html</t>
+  </si>
+  <si>
+    <t>https://lcsc.com/product-detail/chip-resistor-surface-mount_yageo-rc0402fr-071kl_C106235.html</t>
+  </si>
+  <si>
+    <t>https://lcsc.com/product-detail/chip-resistor-surface-mount_yageo-rc0603fr-072k2l_C114662.html</t>
+  </si>
+  <si>
+    <t>https://lcsc.com/product-detail/chip-resistor-surface-mount_yageo-rc0603fr-073k3l_C108078.html</t>
+  </si>
+  <si>
+    <t>https://lcsc.com/product-detail/dc-dc-converters_diodes-ap1509-33sg-13_C151823.html</t>
+  </si>
+  <si>
+    <t>https://lcsc.com/product-detail/rs-485-rs-422-ics_hgsemi-sp3485eim-tr_C519086.html</t>
+  </si>
+  <si>
+    <t>https://lcsc.com/product-detail/transistor-photovoltaic-output-optoisolators_renesas-ps2801c-1-f3-a_C67112.html</t>
+  </si>
+  <si>
+    <t>https://lcsc.com/product-detail/gate-drivers_ti-ucc27517dbvr_C99395.html</t>
   </si>
 </sst>
 </file>
@@ -1044,17 +1110,6 @@
     <xf numFmtId="0" fontId="5" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="top"/>
-      <protection locked="0"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1099,6 +1154,17 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="top"/>
+      <protection locked="0"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -1420,14 +1486,14 @@
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
       <c r="J1" s="2"/>
-      <c r="K1" s="19"/>
-      <c r="L1" s="19"/>
-      <c r="M1" s="19"/>
-      <c r="N1" s="19"/>
-      <c r="O1" s="19"/>
-      <c r="P1" s="19"/>
-      <c r="Q1" s="19"/>
-      <c r="R1" s="19"/>
+      <c r="K1" s="35"/>
+      <c r="L1" s="35"/>
+      <c r="M1" s="35"/>
+      <c r="N1" s="35"/>
+      <c r="O1" s="35"/>
+      <c r="P1" s="35"/>
+      <c r="Q1" s="35"/>
+      <c r="R1" s="35"/>
     </row>
     <row r="2" spans="1:28" ht="15.75" thickBot="1">
       <c r="A2" s="1"/>
@@ -1467,13 +1533,13 @@
       <c r="M2" s="5" t="s">
         <v>175</v>
       </c>
-      <c r="N2" s="29" t="s">
+      <c r="N2" s="26" t="s">
         <v>174</v>
       </c>
       <c r="O2" s="5" t="s">
         <v>173</v>
       </c>
-      <c r="P2" s="32" t="s">
+      <c r="P2" s="29" t="s">
         <v>172</v>
       </c>
       <c r="Q2" s="5" t="s">
@@ -1523,17 +1589,17 @@
         <f>L3*5</f>
         <v>10</v>
       </c>
-      <c r="N3" s="30">
+      <c r="N3" s="27">
         <v>100</v>
       </c>
-      <c r="O3" s="35" t="s">
+      <c r="O3" s="32" t="s">
         <v>207</v>
       </c>
-      <c r="P3" s="33">
+      <c r="P3" s="30">
         <v>3.0999999999999999E-3</v>
       </c>
       <c r="Q3" s="7">
-        <f>P3*N3</f>
+        <f t="shared" ref="Q3:Q17" si="0">P3*N3</f>
         <v>0.31</v>
       </c>
       <c r="R3" s="6"/>
@@ -1541,7 +1607,7 @@
     <row r="4" spans="1:28">
       <c r="A4" s="1"/>
       <c r="B4" s="9">
-        <f t="shared" ref="B4:B30" si="0">ROW(B4) - ROW($B$2)</f>
+        <f t="shared" ref="B4:B30" si="1">ROW(B4) - ROW($B$2)</f>
         <v>2</v>
       </c>
       <c r="C4" s="15" t="s">
@@ -1575,26 +1641,26 @@
         <v>1</v>
       </c>
       <c r="M4" s="12">
-        <f t="shared" ref="M4" si="1">L4*5</f>
+        <f t="shared" ref="M4" si="2">L4*5</f>
         <v>5</v>
       </c>
-      <c r="N4" s="27" t="s">
+      <c r="N4" s="24" t="s">
         <v>182</v>
       </c>
-      <c r="O4" s="35" t="str">
+      <c r="O4" s="32" t="str">
         <f>HYPERLINK(AB4, "LCSC")</f>
         <v>LCSC</v>
       </c>
-      <c r="P4" s="28" t="s">
+      <c r="P4" s="25" t="s">
         <v>187</v>
       </c>
       <c r="Q4" s="13">
-        <f>P4*N4</f>
+        <f t="shared" si="0"/>
         <v>1.3075000000000001</v>
       </c>
       <c r="R4" s="12"/>
-      <c r="V4" s="26"/>
-      <c r="AB4" s="37" t="s">
+      <c r="V4" s="23"/>
+      <c r="AB4" s="34" t="s">
         <v>206</v>
       </c>
     </row>
@@ -1638,30 +1704,30 @@
         <f>L5*5</f>
         <v>10</v>
       </c>
-      <c r="N5" s="30" t="s">
+      <c r="N5" s="27" t="s">
         <v>183</v>
       </c>
-      <c r="O5" s="35" t="str">
-        <f t="shared" ref="O5:O31" si="2">HYPERLINK(AB5, "LCSC")</f>
+      <c r="O5" s="32" t="str">
+        <f t="shared" ref="O5:O31" si="3">HYPERLINK(AB5, "LCSC")</f>
         <v>LCSC</v>
       </c>
-      <c r="P5" s="33" t="s">
+      <c r="P5" s="30" t="s">
         <v>188</v>
       </c>
       <c r="Q5" s="7">
-        <f>P5*N5</f>
+        <f t="shared" si="0"/>
         <v>2.8449999999999998</v>
       </c>
       <c r="R5" s="6"/>
-      <c r="V5" s="26"/>
-      <c r="AB5" s="37" t="s">
-        <v>206</v>
+      <c r="V5" s="23"/>
+      <c r="AB5" s="34" t="s">
+        <v>209</v>
       </c>
     </row>
     <row r="6" spans="1:28">
       <c r="A6" s="1"/>
       <c r="B6" s="9">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>4</v>
       </c>
       <c r="C6" s="15" t="s">
@@ -1695,27 +1761,27 @@
         <v>1</v>
       </c>
       <c r="M6" s="12">
-        <f t="shared" ref="M6" si="3">L6*5</f>
+        <f t="shared" ref="M6" si="4">L6*5</f>
         <v>5</v>
       </c>
-      <c r="N6" s="27" t="s">
+      <c r="N6" s="24" t="s">
         <v>184</v>
       </c>
-      <c r="O6" s="35" t="str">
-        <f t="shared" si="2"/>
+      <c r="O6" s="32" t="str">
+        <f t="shared" si="3"/>
         <v>LCSC</v>
       </c>
-      <c r="P6" s="28" t="s">
+      <c r="P6" s="25" t="s">
         <v>189</v>
       </c>
       <c r="Q6" s="13">
-        <f>P6*N6</f>
+        <f t="shared" si="0"/>
         <v>0.3</v>
       </c>
       <c r="R6" s="12"/>
-      <c r="V6" s="26"/>
-      <c r="AB6" s="37" t="s">
-        <v>206</v>
+      <c r="V6" s="23"/>
+      <c r="AB6" s="34" t="s">
+        <v>210</v>
       </c>
     </row>
     <row r="7" spans="1:28">
@@ -1758,30 +1824,30 @@
         <f>L7*5</f>
         <v>25</v>
       </c>
-      <c r="N7" s="30" t="s">
+      <c r="N7" s="27" t="s">
         <v>184</v>
       </c>
-      <c r="O7" s="35" t="str">
-        <f t="shared" si="2"/>
+      <c r="O7" s="32" t="str">
+        <f t="shared" si="3"/>
         <v>LCSC</v>
       </c>
-      <c r="P7" s="33" t="s">
+      <c r="P7" s="30" t="s">
         <v>190</v>
       </c>
       <c r="Q7" s="7">
-        <f>P7*N7</f>
+        <f t="shared" si="0"/>
         <v>0.16999999999999998</v>
       </c>
       <c r="R7" s="6"/>
-      <c r="V7" s="26"/>
-      <c r="AB7" s="37" t="s">
-        <v>206</v>
+      <c r="V7" s="23"/>
+      <c r="AB7" s="34" t="s">
+        <v>211</v>
       </c>
     </row>
     <row r="8" spans="1:28">
       <c r="A8" s="1"/>
       <c r="B8" s="9">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>6</v>
       </c>
       <c r="C8" s="15" t="s">
@@ -1815,27 +1881,27 @@
         <v>1</v>
       </c>
       <c r="M8" s="12">
-        <f t="shared" ref="M8" si="4">L8*5</f>
+        <f t="shared" ref="M8" si="5">L8*5</f>
         <v>5</v>
       </c>
-      <c r="N8" s="27" t="s">
+      <c r="N8" s="24" t="s">
         <v>183</v>
       </c>
-      <c r="O8" s="35" t="str">
-        <f t="shared" si="2"/>
+      <c r="O8" s="32" t="str">
+        <f t="shared" si="3"/>
         <v>LCSC</v>
       </c>
-      <c r="P8" s="28" t="s">
+      <c r="P8" s="25" t="s">
         <v>191</v>
       </c>
       <c r="Q8" s="13">
-        <f>P8*N8</f>
+        <f t="shared" si="0"/>
         <v>0.36200000000000004</v>
       </c>
       <c r="R8" s="12"/>
-      <c r="V8" s="26"/>
-      <c r="AB8" s="37" t="s">
-        <v>206</v>
+      <c r="V8" s="23"/>
+      <c r="AB8" s="34" t="s">
+        <v>212</v>
       </c>
     </row>
     <row r="9" spans="1:28">
@@ -1878,30 +1944,30 @@
         <f>L9*5</f>
         <v>10</v>
       </c>
-      <c r="N9" s="30" t="s">
+      <c r="N9" s="27" t="s">
         <v>183</v>
       </c>
-      <c r="O9" s="35" t="str">
-        <f t="shared" si="2"/>
+      <c r="O9" s="32" t="str">
+        <f t="shared" si="3"/>
         <v>LCSC</v>
       </c>
-      <c r="P9" s="33" t="s">
+      <c r="P9" s="30" t="s">
         <v>192</v>
       </c>
       <c r="Q9" s="7">
-        <f>P9*N9</f>
+        <f t="shared" si="0"/>
         <v>0.39700000000000002</v>
       </c>
       <c r="R9" s="6"/>
-      <c r="V9" s="26"/>
-      <c r="AB9" s="37" t="s">
-        <v>206</v>
+      <c r="V9" s="23"/>
+      <c r="AB9" s="34" t="s">
+        <v>213</v>
       </c>
     </row>
     <row r="10" spans="1:28" ht="48">
       <c r="A10" s="1"/>
       <c r="B10" s="9">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>8</v>
       </c>
       <c r="C10" s="15" t="s">
@@ -1935,27 +2001,27 @@
         <v>1</v>
       </c>
       <c r="M10" s="12">
-        <f t="shared" ref="M10" si="5">L10*5</f>
+        <f t="shared" ref="M10" si="6">L10*5</f>
         <v>5</v>
       </c>
-      <c r="N10" s="27" t="s">
+      <c r="N10" s="24" t="s">
         <v>182</v>
       </c>
-      <c r="O10" s="35" t="str">
-        <f t="shared" si="2"/>
+      <c r="O10" s="32" t="str">
+        <f t="shared" si="3"/>
         <v>LCSC</v>
       </c>
-      <c r="P10" s="28" t="s">
+      <c r="P10" s="25" t="s">
         <v>193</v>
       </c>
       <c r="Q10" s="13">
-        <f>P10*N10</f>
+        <f t="shared" si="0"/>
         <v>0.99750000000000005</v>
       </c>
       <c r="R10" s="12"/>
-      <c r="V10" s="26"/>
-      <c r="AB10" s="37" t="s">
-        <v>206</v>
+      <c r="V10" s="23"/>
+      <c r="AB10" s="34" t="s">
+        <v>214</v>
       </c>
     </row>
     <row r="11" spans="1:28">
@@ -1998,29 +2064,27 @@
         <f>L11*5</f>
         <v>10</v>
       </c>
-      <c r="N11" s="30" t="s">
+      <c r="N11" s="27" t="s">
         <v>183</v>
       </c>
-      <c r="O11" s="35" t="s">
+      <c r="O11" s="32" t="s">
         <v>208</v>
       </c>
-      <c r="P11" s="33">
+      <c r="P11" s="30">
         <v>1.1399999999999999</v>
       </c>
       <c r="Q11" s="7">
-        <f>P11*N11</f>
+        <f t="shared" si="0"/>
         <v>11.399999999999999</v>
       </c>
       <c r="R11" s="6"/>
-      <c r="V11" s="26"/>
-      <c r="AB11" s="37" t="s">
-        <v>206</v>
-      </c>
+      <c r="V11" s="23"/>
+      <c r="AB11" s="34"/>
     </row>
     <row r="12" spans="1:28" ht="48">
       <c r="A12" s="1"/>
       <c r="B12" s="9">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>10</v>
       </c>
       <c r="C12" s="15" t="s">
@@ -2054,27 +2118,27 @@
         <v>2</v>
       </c>
       <c r="M12" s="12">
-        <f t="shared" ref="M12:M14" si="6">L12*5</f>
+        <f t="shared" ref="M12:M14" si="7">L12*5</f>
         <v>10</v>
       </c>
-      <c r="N12" s="27" t="s">
+      <c r="N12" s="24" t="s">
         <v>185</v>
       </c>
-      <c r="O12" s="35" t="str">
-        <f t="shared" si="2"/>
+      <c r="O12" s="32" t="str">
+        <f t="shared" si="3"/>
         <v>LCSC</v>
       </c>
-      <c r="P12" s="28" t="s">
+      <c r="P12" s="25" t="s">
         <v>194</v>
       </c>
       <c r="Q12" s="13">
-        <f>P12*N12</f>
+        <f t="shared" si="0"/>
         <v>0.61599999999999999</v>
       </c>
       <c r="R12" s="12"/>
-      <c r="V12" s="26"/>
-      <c r="AB12" s="37" t="s">
-        <v>206</v>
+      <c r="V12" s="23"/>
+      <c r="AB12" s="34" t="s">
+        <v>215</v>
       </c>
     </row>
     <row r="13" spans="1:28">
@@ -2114,32 +2178,30 @@
         <v>4</v>
       </c>
       <c r="M13" s="12">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>20</v>
       </c>
-      <c r="N13" s="30">
+      <c r="N13" s="27">
         <v>20</v>
       </c>
-      <c r="O13" s="35" t="s">
+      <c r="O13" s="32" t="s">
         <v>208</v>
       </c>
-      <c r="P13" s="33">
+      <c r="P13" s="30">
         <v>0.63</v>
       </c>
       <c r="Q13" s="7">
-        <f>P13*N13</f>
+        <f t="shared" si="0"/>
         <v>12.6</v>
       </c>
       <c r="R13" s="6"/>
-      <c r="V13" s="26"/>
-      <c r="AB13" s="37" t="s">
-        <v>206</v>
-      </c>
+      <c r="V13" s="23"/>
+      <c r="AB13" s="34"/>
     </row>
     <row r="14" spans="1:28">
       <c r="A14" s="1"/>
       <c r="B14" s="9">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>12</v>
       </c>
       <c r="C14" s="15" t="s">
@@ -2173,27 +2235,25 @@
         <v>3</v>
       </c>
       <c r="M14" s="12">
-        <f t="shared" si="6"/>
+        <f t="shared" si="7"/>
         <v>15</v>
       </c>
-      <c r="N14" s="27">
+      <c r="N14" s="24">
         <v>15</v>
       </c>
-      <c r="O14" s="35" t="s">
+      <c r="O14" s="32" t="s">
         <v>208</v>
       </c>
-      <c r="P14" s="28">
+      <c r="P14" s="25">
         <v>0.75</v>
       </c>
       <c r="Q14" s="13">
-        <f>P14*N14</f>
+        <f t="shared" si="0"/>
         <v>11.25</v>
       </c>
       <c r="R14" s="12"/>
-      <c r="V14" s="26"/>
-      <c r="AB14" s="37" t="s">
-        <v>206</v>
-      </c>
+      <c r="V14" s="23"/>
+      <c r="AB14" s="34"/>
     </row>
     <row r="15" spans="1:28" ht="24">
       <c r="A15" s="1"/>
@@ -2235,30 +2295,30 @@
         <f>L15*5</f>
         <v>5</v>
       </c>
-      <c r="N15" s="30" t="s">
+      <c r="N15" s="27" t="s">
         <v>182</v>
       </c>
-      <c r="O15" s="35" t="str">
-        <f t="shared" si="2"/>
+      <c r="O15" s="32" t="str">
+        <f t="shared" si="3"/>
         <v>LCSC</v>
       </c>
-      <c r="P15" s="33" t="s">
+      <c r="P15" s="30" t="s">
         <v>195</v>
       </c>
       <c r="Q15" s="7">
-        <f>P15*N15</f>
+        <f t="shared" si="0"/>
         <v>4.6985000000000001</v>
       </c>
       <c r="R15" s="6"/>
-      <c r="V15" s="26"/>
-      <c r="AB15" s="37" t="s">
-        <v>206</v>
+      <c r="V15" s="23"/>
+      <c r="AB15" s="34" t="s">
+        <v>216</v>
       </c>
     </row>
     <row r="16" spans="1:28" ht="24">
       <c r="A16" s="1"/>
       <c r="B16" s="9">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>14</v>
       </c>
       <c r="C16" s="15" t="s">
@@ -2292,27 +2352,27 @@
         <v>3</v>
       </c>
       <c r="M16" s="12">
-        <f t="shared" ref="M16" si="7">L16*5</f>
+        <f t="shared" ref="M16" si="8">L16*5</f>
         <v>15</v>
       </c>
-      <c r="N16" s="27" t="s">
+      <c r="N16" s="24" t="s">
         <v>185</v>
       </c>
-      <c r="O16" s="35" t="str">
-        <f t="shared" si="2"/>
+      <c r="O16" s="32" t="str">
+        <f t="shared" si="3"/>
         <v>LCSC</v>
       </c>
-      <c r="P16" s="28" t="s">
+      <c r="P16" s="25" t="s">
         <v>196</v>
       </c>
       <c r="Q16" s="13">
-        <f>P16*N16</f>
+        <f t="shared" si="0"/>
         <v>1.274</v>
       </c>
       <c r="R16" s="12"/>
-      <c r="V16" s="26"/>
-      <c r="AB16" s="37" t="s">
-        <v>206</v>
+      <c r="V16" s="23"/>
+      <c r="AB16" s="34" t="s">
+        <v>217</v>
       </c>
     </row>
     <row r="17" spans="1:28" ht="24">
@@ -2355,85 +2415,85 @@
         <f>L17*5</f>
         <v>65</v>
       </c>
-      <c r="N17" s="30" t="s">
+      <c r="N17" s="27" t="s">
         <v>184</v>
       </c>
-      <c r="O17" s="35" t="str">
-        <f t="shared" si="2"/>
+      <c r="O17" s="32" t="str">
+        <f t="shared" si="3"/>
         <v>LCSC</v>
       </c>
-      <c r="P17" s="33" t="s">
+      <c r="P17" s="30" t="s">
         <v>197</v>
       </c>
       <c r="Q17" s="7">
-        <f>P17*N17</f>
+        <f t="shared" si="0"/>
         <v>0.11</v>
       </c>
       <c r="R17" s="6"/>
-      <c r="V17" s="26"/>
-      <c r="AB17" s="37" t="s">
-        <v>206</v>
+      <c r="V17" s="23"/>
+      <c r="AB17" s="34" t="s">
+        <v>218</v>
       </c>
     </row>
     <row r="18" spans="1:28">
       <c r="A18" s="1"/>
       <c r="B18" s="9">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>16</v>
       </c>
       <c r="C18" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="D18" s="22" t="s">
+      <c r="D18" s="19" t="s">
         <v>31</v>
       </c>
-      <c r="E18" s="22" t="s">
+      <c r="E18" s="19" t="s">
         <v>59</v>
       </c>
-      <c r="F18" s="22" t="s">
+      <c r="F18" s="19" t="s">
         <v>86</v>
       </c>
-      <c r="G18" s="22" t="s">
+      <c r="G18" s="19" t="s">
         <v>104</v>
       </c>
-      <c r="H18" s="22" t="s">
+      <c r="H18" s="19" t="s">
         <v>117</v>
       </c>
       <c r="I18" s="6" t="s">
         <v>179</v>
       </c>
-      <c r="J18" s="22" t="s">
+      <c r="J18" s="19" t="s">
         <v>180</v>
       </c>
-      <c r="K18" s="23" t="s">
+      <c r="K18" s="20" t="s">
         <v>162</v>
       </c>
-      <c r="L18" s="22">
+      <c r="L18" s="19">
         <v>1</v>
       </c>
-      <c r="M18" s="22">
-        <f t="shared" ref="M18" si="8">L18*5</f>
+      <c r="M18" s="19">
+        <f t="shared" ref="M18" si="9">L18*5</f>
         <v>5</v>
       </c>
-      <c r="N18" s="31" t="s">
+      <c r="N18" s="28" t="s">
         <v>184</v>
       </c>
-      <c r="O18" s="35" t="str">
-        <f t="shared" si="2"/>
+      <c r="O18" s="32" t="str">
+        <f t="shared" si="3"/>
         <v>LCSC</v>
       </c>
-      <c r="P18" s="34" t="s">
-        <v>179</v>
-      </c>
-      <c r="Q18" s="24" t="s">
-        <v>179</v>
-      </c>
-      <c r="R18" s="25" t="s">
+      <c r="P18" s="31" t="s">
+        <v>179</v>
+      </c>
+      <c r="Q18" s="21" t="s">
+        <v>179</v>
+      </c>
+      <c r="R18" s="22" t="s">
         <v>181</v>
       </c>
-      <c r="V18" s="26"/>
-      <c r="AB18" s="37" t="s">
-        <v>206</v>
+      <c r="V18" s="23"/>
+      <c r="AB18" s="34" t="s">
+        <v>219</v>
       </c>
     </row>
     <row r="19" spans="1:28">
@@ -2476,14 +2536,14 @@
         <f>L19*5</f>
         <v>5</v>
       </c>
-      <c r="N19" s="30" t="s">
+      <c r="N19" s="27" t="s">
         <v>184</v>
       </c>
-      <c r="O19" s="35" t="str">
-        <f t="shared" si="2"/>
+      <c r="O19" s="32" t="str">
+        <f t="shared" si="3"/>
         <v>LCSC</v>
       </c>
-      <c r="P19" s="33" t="s">
+      <c r="P19" s="30" t="s">
         <v>198</v>
       </c>
       <c r="Q19" s="7">
@@ -2491,15 +2551,15 @@
         <v>0.31</v>
       </c>
       <c r="R19" s="6"/>
-      <c r="V19" s="26"/>
-      <c r="AB19" s="37" t="s">
-        <v>206</v>
+      <c r="V19" s="23"/>
+      <c r="AB19" s="34" t="s">
+        <v>219</v>
       </c>
     </row>
     <row r="20" spans="1:28">
       <c r="A20" s="1"/>
       <c r="B20" s="9">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>18</v>
       </c>
       <c r="C20" s="15" t="s">
@@ -2533,17 +2593,17 @@
         <v>4</v>
       </c>
       <c r="M20" s="12">
-        <f t="shared" ref="M20" si="9">L20*5</f>
+        <f t="shared" ref="M20" si="10">L20*5</f>
         <v>20</v>
       </c>
-      <c r="N20" s="27" t="s">
+      <c r="N20" s="24" t="s">
         <v>184</v>
       </c>
-      <c r="O20" s="35" t="str">
-        <f t="shared" si="2"/>
+      <c r="O20" s="32" t="str">
+        <f t="shared" si="3"/>
         <v>LCSC</v>
       </c>
-      <c r="P20" s="28" t="s">
+      <c r="P20" s="25" t="s">
         <v>199</v>
       </c>
       <c r="Q20" s="13">
@@ -2551,9 +2611,9 @@
         <v>0.06</v>
       </c>
       <c r="R20" s="12"/>
-      <c r="V20" s="26"/>
-      <c r="AB20" s="37" t="s">
-        <v>206</v>
+      <c r="V20" s="23"/>
+      <c r="AB20" s="34" t="s">
+        <v>220</v>
       </c>
     </row>
     <row r="21" spans="1:28">
@@ -2596,14 +2656,14 @@
         <f>L21*5</f>
         <v>20</v>
       </c>
-      <c r="N21" s="30" t="s">
+      <c r="N21" s="27" t="s">
         <v>184</v>
       </c>
-      <c r="O21" s="35" t="str">
-        <f t="shared" si="2"/>
+      <c r="O21" s="32" t="str">
+        <f t="shared" si="3"/>
         <v>LCSC</v>
       </c>
-      <c r="P21" s="33" t="s">
+      <c r="P21" s="30" t="s">
         <v>199</v>
       </c>
       <c r="Q21" s="7">
@@ -2611,15 +2671,15 @@
         <v>0.06</v>
       </c>
       <c r="R21" s="6"/>
-      <c r="V21" s="26"/>
-      <c r="AB21" s="37" t="s">
-        <v>206</v>
+      <c r="V21" s="23"/>
+      <c r="AB21" s="34" t="s">
+        <v>221</v>
       </c>
     </row>
     <row r="22" spans="1:28">
       <c r="A22" s="1"/>
       <c r="B22" s="9">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>20</v>
       </c>
       <c r="C22" s="15" t="s">
@@ -2653,17 +2713,17 @@
         <v>2</v>
       </c>
       <c r="M22" s="12">
-        <f t="shared" ref="M22" si="10">L22*5</f>
+        <f t="shared" ref="M22" si="11">L22*5</f>
         <v>10</v>
       </c>
-      <c r="N22" s="27" t="s">
+      <c r="N22" s="24" t="s">
         <v>184</v>
       </c>
-      <c r="O22" s="35" t="str">
-        <f t="shared" si="2"/>
+      <c r="O22" s="32" t="str">
+        <f t="shared" si="3"/>
         <v>LCSC</v>
       </c>
-      <c r="P22" s="28" t="s">
+      <c r="P22" s="25" t="s">
         <v>200</v>
       </c>
       <c r="Q22" s="13">
@@ -2671,9 +2731,9 @@
         <v>0.12</v>
       </c>
       <c r="R22" s="12"/>
-      <c r="V22" s="26"/>
-      <c r="AB22" s="37" t="s">
-        <v>206</v>
+      <c r="V22" s="23"/>
+      <c r="AB22" s="34" t="s">
+        <v>222</v>
       </c>
     </row>
     <row r="23" spans="1:28">
@@ -2685,62 +2745,62 @@
       <c r="C23" s="14" t="s">
         <v>12</v>
       </c>
-      <c r="D23" s="22" t="s">
+      <c r="D23" s="19" t="s">
         <v>36</v>
       </c>
-      <c r="E23" s="22" t="s">
+      <c r="E23" s="19" t="s">
         <v>60</v>
       </c>
-      <c r="F23" s="22" t="s">
+      <c r="F23" s="19" t="s">
         <v>87</v>
       </c>
-      <c r="G23" s="22" t="s">
+      <c r="G23" s="19" t="s">
         <v>105</v>
       </c>
-      <c r="H23" s="22" t="s">
+      <c r="H23" s="19" t="s">
         <v>117</v>
       </c>
       <c r="I23" s="6" t="s">
         <v>179</v>
       </c>
-      <c r="J23" s="22" t="s">
+      <c r="J23" s="19" t="s">
         <v>146</v>
       </c>
-      <c r="K23" s="23" t="s">
+      <c r="K23" s="20" t="s">
         <v>162</v>
       </c>
-      <c r="L23" s="22">
+      <c r="L23" s="19">
         <v>2</v>
       </c>
-      <c r="M23" s="22">
+      <c r="M23" s="19">
         <f>L23*5</f>
         <v>10</v>
       </c>
-      <c r="N23" s="31" t="s">
+      <c r="N23" s="28" t="s">
         <v>184</v>
       </c>
-      <c r="O23" s="35" t="str">
-        <f t="shared" si="2"/>
+      <c r="O23" s="32" t="str">
+        <f t="shared" si="3"/>
         <v>LCSC</v>
       </c>
-      <c r="P23" s="34" t="s">
-        <v>179</v>
-      </c>
-      <c r="Q23" s="24" t="s">
-        <v>179</v>
-      </c>
-      <c r="R23" s="25" t="s">
+      <c r="P23" s="31" t="s">
+        <v>179</v>
+      </c>
+      <c r="Q23" s="21" t="s">
+        <v>179</v>
+      </c>
+      <c r="R23" s="22" t="s">
         <v>181</v>
       </c>
-      <c r="V23" s="26"/>
-      <c r="AB23" s="37" t="s">
-        <v>206</v>
+      <c r="V23" s="23"/>
+      <c r="AB23" s="34" t="s">
+        <v>220</v>
       </c>
     </row>
     <row r="24" spans="1:28">
       <c r="A24" s="1"/>
       <c r="B24" s="9">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>22</v>
       </c>
       <c r="C24" s="14" t="s">
@@ -2774,27 +2834,27 @@
         <v>3</v>
       </c>
       <c r="M24" s="12">
-        <f t="shared" ref="M24" si="11">L24*5</f>
+        <f t="shared" ref="M24" si="12">L24*5</f>
         <v>15</v>
       </c>
-      <c r="N24" s="27" t="s">
+      <c r="N24" s="24" t="s">
         <v>186</v>
       </c>
-      <c r="O24" s="35" t="str">
-        <f t="shared" si="2"/>
+      <c r="O24" s="32" t="str">
+        <f t="shared" si="3"/>
         <v>LCSC</v>
       </c>
-      <c r="P24" s="28" t="s">
+      <c r="P24" s="25" t="s">
         <v>201</v>
       </c>
       <c r="Q24" s="13">
-        <f>P24*N24</f>
+        <f t="shared" ref="Q24:Q31" si="13">P24*N24</f>
         <v>1.458</v>
       </c>
       <c r="R24" s="12"/>
-      <c r="V24" s="26"/>
-      <c r="AB24" s="37" t="s">
-        <v>206</v>
+      <c r="V24" s="23"/>
+      <c r="AB24" s="34" t="s">
+        <v>223</v>
       </c>
     </row>
     <row r="25" spans="1:28">
@@ -2837,30 +2897,30 @@
         <f>L25*5</f>
         <v>15</v>
       </c>
-      <c r="N25" s="30" t="s">
+      <c r="N25" s="27" t="s">
         <v>184</v>
       </c>
-      <c r="O25" s="35" t="str">
-        <f t="shared" si="2"/>
+      <c r="O25" s="32" t="str">
+        <f t="shared" si="3"/>
         <v>LCSC</v>
       </c>
-      <c r="P25" s="33" t="s">
+      <c r="P25" s="30" t="s">
         <v>199</v>
       </c>
       <c r="Q25" s="7">
-        <f>P25*N25</f>
+        <f t="shared" si="13"/>
         <v>0.06</v>
       </c>
       <c r="R25" s="6"/>
-      <c r="V25" s="26"/>
-      <c r="AB25" s="37" t="s">
-        <v>206</v>
+      <c r="V25" s="23"/>
+      <c r="AB25" s="34" t="s">
+        <v>224</v>
       </c>
     </row>
     <row r="26" spans="1:28">
       <c r="A26" s="1"/>
       <c r="B26" s="9">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>24</v>
       </c>
       <c r="C26" s="15" t="s">
@@ -2894,27 +2954,27 @@
         <v>3</v>
       </c>
       <c r="M26" s="12">
-        <f t="shared" ref="M26" si="12">L26*5</f>
+        <f t="shared" ref="M26" si="14">L26*5</f>
         <v>15</v>
       </c>
-      <c r="N26" s="27" t="s">
+      <c r="N26" s="24" t="s">
         <v>184</v>
       </c>
-      <c r="O26" s="35" t="str">
-        <f t="shared" si="2"/>
+      <c r="O26" s="32" t="str">
+        <f t="shared" si="3"/>
         <v>LCSC</v>
       </c>
-      <c r="P26" s="28" t="s">
+      <c r="P26" s="25" t="s">
         <v>200</v>
       </c>
       <c r="Q26" s="13">
-        <f>P26*N26</f>
+        <f t="shared" si="13"/>
         <v>0.12</v>
       </c>
       <c r="R26" s="12"/>
-      <c r="V26" s="26"/>
-      <c r="AB26" s="37" t="s">
-        <v>206</v>
+      <c r="V26" s="23"/>
+      <c r="AB26" s="34" t="s">
+        <v>225</v>
       </c>
     </row>
     <row r="27" spans="1:28">
@@ -2957,30 +3017,30 @@
         <f>L27*5</f>
         <v>15</v>
       </c>
-      <c r="N27" s="30" t="s">
+      <c r="N27" s="27" t="s">
         <v>184</v>
       </c>
-      <c r="O27" s="35" t="str">
-        <f t="shared" si="2"/>
+      <c r="O27" s="32" t="str">
+        <f t="shared" si="3"/>
         <v>LCSC</v>
       </c>
-      <c r="P27" s="33" t="s">
+      <c r="P27" s="30" t="s">
         <v>200</v>
       </c>
       <c r="Q27" s="7">
-        <f>P27*N27</f>
+        <f t="shared" si="13"/>
         <v>0.12</v>
       </c>
       <c r="R27" s="6"/>
-      <c r="V27" s="26"/>
-      <c r="AB27" s="37" t="s">
-        <v>206</v>
+      <c r="V27" s="23"/>
+      <c r="AB27" s="34" t="s">
+        <v>226</v>
       </c>
     </row>
     <row r="28" spans="1:28">
       <c r="A28" s="1"/>
       <c r="B28" s="9">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>26</v>
       </c>
       <c r="C28" s="15" t="s">
@@ -3014,27 +3074,27 @@
         <v>1</v>
       </c>
       <c r="M28" s="12">
-        <f t="shared" ref="M28" si="13">L28*5</f>
+        <f t="shared" ref="M28" si="15">L28*5</f>
         <v>5</v>
       </c>
-      <c r="N28" s="27" t="s">
+      <c r="N28" s="24" t="s">
         <v>182</v>
       </c>
-      <c r="O28" s="35" t="str">
-        <f t="shared" si="2"/>
+      <c r="O28" s="32" t="str">
+        <f t="shared" si="3"/>
         <v>LCSC</v>
       </c>
-      <c r="P28" s="28" t="s">
+      <c r="P28" s="25" t="s">
         <v>202</v>
       </c>
       <c r="Q28" s="13">
-        <f>P28*N28</f>
+        <f t="shared" si="13"/>
         <v>2.3445</v>
       </c>
       <c r="R28" s="12"/>
-      <c r="V28" s="26"/>
-      <c r="AB28" s="37" t="s">
-        <v>206</v>
+      <c r="V28" s="23"/>
+      <c r="AB28" s="34" t="s">
+        <v>227</v>
       </c>
     </row>
     <row r="29" spans="1:28">
@@ -3077,30 +3137,30 @@
         <f>L29*5</f>
         <v>10</v>
       </c>
-      <c r="N29" s="30" t="s">
+      <c r="N29" s="27" t="s">
         <v>183</v>
       </c>
-      <c r="O29" s="35" t="str">
-        <f t="shared" si="2"/>
+      <c r="O29" s="32" t="str">
+        <f t="shared" si="3"/>
         <v>LCSC</v>
       </c>
-      <c r="P29" s="33" t="s">
+      <c r="P29" s="30" t="s">
         <v>203</v>
       </c>
       <c r="Q29" s="7">
-        <f>P29*N29</f>
+        <f t="shared" si="13"/>
         <v>2.4220000000000002</v>
       </c>
       <c r="R29" s="6"/>
-      <c r="V29" s="26"/>
-      <c r="AB29" s="37" t="s">
-        <v>206</v>
+      <c r="V29" s="23"/>
+      <c r="AB29" s="34" t="s">
+        <v>228</v>
       </c>
     </row>
     <row r="30" spans="1:28" ht="36">
       <c r="A30" s="1"/>
       <c r="B30" s="9">
-        <f t="shared" si="0"/>
+        <f t="shared" si="1"/>
         <v>28</v>
       </c>
       <c r="C30" s="14" t="s">
@@ -3134,27 +3194,27 @@
         <v>3</v>
       </c>
       <c r="M30" s="12">
-        <f t="shared" ref="M30" si="14">L30*5</f>
+        <f t="shared" ref="M30" si="16">L30*5</f>
         <v>15</v>
       </c>
-      <c r="N30" s="27" t="s">
+      <c r="N30" s="24" t="s">
         <v>186</v>
       </c>
-      <c r="O30" s="35" t="str">
-        <f t="shared" si="2"/>
+      <c r="O30" s="32" t="str">
+        <f t="shared" si="3"/>
         <v>LCSC</v>
       </c>
-      <c r="P30" s="28" t="s">
+      <c r="P30" s="25" t="s">
         <v>204</v>
       </c>
       <c r="Q30" s="13">
-        <f>P30*N30</f>
+        <f t="shared" si="13"/>
         <v>4.0875000000000004</v>
       </c>
       <c r="R30" s="12"/>
-      <c r="V30" s="26"/>
-      <c r="AB30" s="37" t="s">
-        <v>206</v>
+      <c r="V30" s="23"/>
+      <c r="AB30" s="34" t="s">
+        <v>229</v>
       </c>
     </row>
     <row r="31" spans="1:28" ht="15.75" thickBot="1">
@@ -3197,24 +3257,24 @@
         <f>L31*5</f>
         <v>15</v>
       </c>
-      <c r="N31" s="30" t="s">
+      <c r="N31" s="27" t="s">
         <v>186</v>
       </c>
-      <c r="O31" s="36" t="str">
-        <f t="shared" si="2"/>
+      <c r="O31" s="33" t="str">
+        <f t="shared" si="3"/>
         <v>LCSC</v>
       </c>
-      <c r="P31" s="33" t="s">
+      <c r="P31" s="30" t="s">
         <v>205</v>
       </c>
       <c r="Q31" s="7">
-        <f>P31*N31</f>
+        <f t="shared" si="13"/>
         <v>3.1110000000000002</v>
       </c>
       <c r="R31" s="6"/>
-      <c r="V31" s="26"/>
-      <c r="AB31" s="37" t="s">
-        <v>206</v>
+      <c r="V31" s="23"/>
+      <c r="AB31" s="34" t="s">
+        <v>230</v>
       </c>
     </row>
     <row r="32" spans="1:28" ht="19.5" thickBot="1">
@@ -3231,11 +3291,11 @@
       <c r="K32" s="1"/>
       <c r="L32" s="1"/>
       <c r="M32" s="1"/>
-      <c r="N32" s="20" t="s">
+      <c r="N32" s="36" t="s">
         <v>1</v>
       </c>
-      <c r="O32" s="21"/>
-      <c r="P32" s="21"/>
+      <c r="O32" s="37"/>
+      <c r="P32" s="37"/>
       <c r="Q32" s="10">
         <f>SUM(Q3:Q31)</f>
         <v>62.910499999999999</v>
@@ -3256,11 +3316,11 @@
       <c r="K33" s="1"/>
       <c r="L33" s="1"/>
       <c r="M33" s="1"/>
-      <c r="N33" s="20" t="s">
+      <c r="N33" s="36" t="s">
         <v>2</v>
       </c>
-      <c r="O33" s="21"/>
-      <c r="P33" s="21"/>
+      <c r="O33" s="37"/>
+      <c r="P33" s="37"/>
       <c r="Q33" s="11">
         <f>Q32/5</f>
         <v>12.582100000000001</v>
@@ -3277,14 +3337,37 @@
     <mergeCell ref="N33:P33"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="AB4" r:id="rId1" display="url"/>
-    <hyperlink ref="AB5:AB31" r:id="rId2" display="url"/>
-    <hyperlink ref="O11" r:id="rId3"/>
-    <hyperlink ref="O13" r:id="rId4"/>
-    <hyperlink ref="O14" r:id="rId5"/>
-    <hyperlink ref="O3" r:id="rId6"/>
+    <hyperlink ref="O11" r:id="rId1"/>
+    <hyperlink ref="O13" r:id="rId2"/>
+    <hyperlink ref="O14" r:id="rId3"/>
+    <hyperlink ref="O3" r:id="rId4"/>
+    <hyperlink ref="AB4" r:id="rId5" display="url"/>
+    <hyperlink ref="AB5" r:id="rId6" display="url"/>
+    <hyperlink ref="AB6" r:id="rId7" display="url"/>
+    <hyperlink ref="AB7" r:id="rId8" display="url"/>
+    <hyperlink ref="AB8" r:id="rId9" display="url"/>
+    <hyperlink ref="AB9" r:id="rId10" display="url"/>
+    <hyperlink ref="AB10" r:id="rId11" display="url"/>
+    <hyperlink ref="AB12" r:id="rId12" display="url"/>
+    <hyperlink ref="AB15" r:id="rId13" display="url"/>
+    <hyperlink ref="AB16" r:id="rId14" display="url"/>
+    <hyperlink ref="AB17" r:id="rId15" display="url"/>
+    <hyperlink ref="AB18" r:id="rId16" display="url"/>
+    <hyperlink ref="AB19" r:id="rId17" display="url"/>
+    <hyperlink ref="AB20" r:id="rId18" display="url"/>
+    <hyperlink ref="AB21" r:id="rId19" display="url"/>
+    <hyperlink ref="AB22" r:id="rId20" display="url"/>
+    <hyperlink ref="AB23" r:id="rId21" display="url"/>
+    <hyperlink ref="AB24" r:id="rId22" display="url"/>
+    <hyperlink ref="AB25" r:id="rId23" display="url"/>
+    <hyperlink ref="AB26" r:id="rId24" display="url"/>
+    <hyperlink ref="AB27" r:id="rId25" display="url"/>
+    <hyperlink ref="AB28" r:id="rId26" display="url"/>
+    <hyperlink ref="AB29" r:id="rId27" display="url"/>
+    <hyperlink ref="AB30" r:id="rId28" display="url"/>
+    <hyperlink ref="AB31" r:id="rId29" display="url"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId7"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId30"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
BB_Board 100 Pcs BOM Added.
</commit_message>
<xml_diff>
--- a/Design-Files/BB_Production/BOM/BOM-With-Price_BB_Production.xlsx
+++ b/Design-Files/BB_Production/BOM/BOM-With-Price_BB_Production.xlsx
@@ -13,13 +13,14 @@
   </bookViews>
   <sheets>
     <sheet name="5 Boards" sheetId="1" r:id="rId1"/>
+    <sheet name="100 Boards" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="162913"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="364" uniqueCount="231">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="694" uniqueCount="252">
   <si>
     <t>#</t>
   </si>
@@ -712,6 +713,69 @@
   </si>
   <si>
     <t>https://lcsc.com/product-detail/gate-drivers_ti-ucc27517dbvr_C99395.html</t>
+  </si>
+  <si>
+    <t>Quantity (100 Boards)</t>
+  </si>
+  <si>
+    <t>MOQ (100 Boards)</t>
+  </si>
+  <si>
+    <t>Unit Cost (100 Boards)</t>
+  </si>
+  <si>
+    <t>Total Cost (100 Boards)</t>
+  </si>
+  <si>
+    <t>0.1524</t>
+  </si>
+  <si>
+    <t>0.1887</t>
+  </si>
+  <si>
+    <t>0.0284</t>
+  </si>
+  <si>
+    <t>0.1572</t>
+  </si>
+  <si>
+    <t>0.0244</t>
+  </si>
+  <si>
+    <t>0.5998</t>
+  </si>
+  <si>
+    <t>0.0441</t>
+  </si>
+  <si>
+    <t>0.0008</t>
+  </si>
+  <si>
+    <t>0.0377</t>
+  </si>
+  <si>
+    <t>0.2767</t>
+  </si>
+  <si>
+    <t>0.1703</t>
+  </si>
+  <si>
+    <t>0.2018</t>
+  </si>
+  <si>
+    <t>0.1398</t>
+  </si>
+  <si>
+    <t>300</t>
+  </si>
+  <si>
+    <t>1300</t>
+  </si>
+  <si>
+    <t>400</t>
+  </si>
+  <si>
+    <t>200</t>
   </si>
 </sst>
 </file>
@@ -1060,7 +1124,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -1154,6 +1218,18 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1486,14 +1562,14 @@
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
       <c r="J1" s="2"/>
-      <c r="K1" s="35"/>
-      <c r="L1" s="35"/>
-      <c r="M1" s="35"/>
-      <c r="N1" s="35"/>
-      <c r="O1" s="35"/>
-      <c r="P1" s="35"/>
-      <c r="Q1" s="35"/>
-      <c r="R1" s="35"/>
+      <c r="K1" s="39"/>
+      <c r="L1" s="39"/>
+      <c r="M1" s="39"/>
+      <c r="N1" s="39"/>
+      <c r="O1" s="39"/>
+      <c r="P1" s="39"/>
+      <c r="Q1" s="39"/>
+      <c r="R1" s="39"/>
     </row>
     <row r="2" spans="1:28" ht="15.75" thickBot="1">
       <c r="A2" s="1"/>
@@ -3291,11 +3367,11 @@
       <c r="K32" s="1"/>
       <c r="L32" s="1"/>
       <c r="M32" s="1"/>
-      <c r="N32" s="36" t="s">
+      <c r="N32" s="40" t="s">
         <v>1</v>
       </c>
-      <c r="O32" s="37"/>
-      <c r="P32" s="37"/>
+      <c r="O32" s="41"/>
+      <c r="P32" s="41"/>
       <c r="Q32" s="10">
         <f>SUM(Q3:Q31)</f>
         <v>62.910499999999999</v>
@@ -3316,11 +3392,11 @@
       <c r="K33" s="1"/>
       <c r="L33" s="1"/>
       <c r="M33" s="1"/>
-      <c r="N33" s="36" t="s">
+      <c r="N33" s="40" t="s">
         <v>2</v>
       </c>
-      <c r="O33" s="37"/>
-      <c r="P33" s="37"/>
+      <c r="O33" s="41"/>
+      <c r="P33" s="41"/>
       <c r="Q33" s="11">
         <f>Q32/5</f>
         <v>12.582100000000001</v>
@@ -3370,4 +3446,1790 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId30"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:R33"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="2" max="2" width="3" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.85546875" customWidth="1"/>
+    <col min="4" max="4" width="14.140625" customWidth="1"/>
+    <col min="5" max="5" width="27.85546875" customWidth="1"/>
+    <col min="6" max="6" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="25.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.28515625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="21.5703125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="6.140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8.7109375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="20.28515625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="17.28515625" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="7.7109375" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="20.7109375" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="21.42578125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="9" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:18" ht="15.75" thickBot="1">
+      <c r="A1" s="1"/>
+      <c r="B1" s="3"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
+      <c r="J1" s="2"/>
+      <c r="K1" s="39"/>
+      <c r="L1" s="39"/>
+      <c r="M1" s="39"/>
+      <c r="N1" s="39"/>
+      <c r="O1" s="39"/>
+      <c r="P1" s="39"/>
+      <c r="Q1" s="39"/>
+      <c r="R1" s="39"/>
+    </row>
+    <row r="2" spans="1:18" ht="15.75" thickBot="1">
+      <c r="A2" s="1"/>
+      <c r="B2" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="5" t="s">
+        <v>3</v>
+      </c>
+      <c r="D2" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="E2" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="F2" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="G2" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="H2" s="5" t="s">
+        <v>116</v>
+      </c>
+      <c r="I2" s="5" t="s">
+        <v>176</v>
+      </c>
+      <c r="J2" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="K2" s="5" t="s">
+        <v>177</v>
+      </c>
+      <c r="L2" s="5" t="s">
+        <v>169</v>
+      </c>
+      <c r="M2" s="5" t="s">
+        <v>231</v>
+      </c>
+      <c r="N2" s="26" t="s">
+        <v>232</v>
+      </c>
+      <c r="O2" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="P2" s="29" t="s">
+        <v>233</v>
+      </c>
+      <c r="Q2" s="5" t="s">
+        <v>234</v>
+      </c>
+      <c r="R2" s="5" t="s">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="3" spans="1:18" s="37" customFormat="1">
+      <c r="A3" s="35"/>
+      <c r="B3" s="8">
+        <f>ROW(B3) - ROW($B$2)</f>
+        <v>1</v>
+      </c>
+      <c r="C3" s="14" t="s">
+        <v>4</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="F3" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="G3" s="6" t="s">
+        <v>94</v>
+      </c>
+      <c r="H3" s="6" t="s">
+        <v>117</v>
+      </c>
+      <c r="I3" s="6" t="s">
+        <v>179</v>
+      </c>
+      <c r="J3" s="6" t="s">
+        <v>134</v>
+      </c>
+      <c r="K3" s="17" t="s">
+        <v>157</v>
+      </c>
+      <c r="L3" s="6">
+        <v>2</v>
+      </c>
+      <c r="M3" s="6">
+        <f>L3*100</f>
+        <v>200</v>
+      </c>
+      <c r="N3" s="27">
+        <v>300</v>
+      </c>
+      <c r="O3" s="36" t="s">
+        <v>207</v>
+      </c>
+      <c r="P3" s="30">
+        <v>3.0999999999999999E-3</v>
+      </c>
+      <c r="Q3" s="7">
+        <f t="shared" ref="Q3:Q17" si="0">P3*N3</f>
+        <v>0.92999999999999994</v>
+      </c>
+      <c r="R3" s="6"/>
+    </row>
+    <row r="4" spans="1:18" s="37" customFormat="1">
+      <c r="A4" s="35"/>
+      <c r="B4" s="9">
+        <f t="shared" ref="B4:B30" si="1">ROW(B4) - ROW($B$2)</f>
+        <v>2</v>
+      </c>
+      <c r="C4" s="15" t="s">
+        <v>4</v>
+      </c>
+      <c r="D4" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="E4" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="F4" s="12" t="s">
+        <v>73</v>
+      </c>
+      <c r="G4" s="12" t="s">
+        <v>95</v>
+      </c>
+      <c r="H4" s="12" t="s">
+        <v>118</v>
+      </c>
+      <c r="I4" s="6" t="s">
+        <v>179</v>
+      </c>
+      <c r="J4" s="12" t="s">
+        <v>135</v>
+      </c>
+      <c r="K4" s="18" t="s">
+        <v>158</v>
+      </c>
+      <c r="L4" s="12">
+        <v>1</v>
+      </c>
+      <c r="M4" s="6">
+        <f t="shared" ref="M4:M31" si="2">L4*100</f>
+        <v>100</v>
+      </c>
+      <c r="N4" s="24">
+        <v>105</v>
+      </c>
+      <c r="O4" s="36" t="str">
+        <f>HYPERLINK(AB4, "LCSC")</f>
+        <v>LCSC</v>
+      </c>
+      <c r="P4" s="25" t="s">
+        <v>235</v>
+      </c>
+      <c r="Q4" s="13">
+        <f t="shared" si="0"/>
+        <v>16.002000000000002</v>
+      </c>
+      <c r="R4" s="12"/>
+    </row>
+    <row r="5" spans="1:18" s="37" customFormat="1">
+      <c r="A5" s="35"/>
+      <c r="B5" s="8">
+        <f>ROW(B5) - ROW($B$2)</f>
+        <v>3</v>
+      </c>
+      <c r="C5" s="14" t="s">
+        <v>4</v>
+      </c>
+      <c r="D5" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="E5" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="F5" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="G5" s="6" t="s">
+        <v>96</v>
+      </c>
+      <c r="H5" s="6" t="s">
+        <v>119</v>
+      </c>
+      <c r="I5" s="6" t="s">
+        <v>179</v>
+      </c>
+      <c r="J5" s="6" t="s">
+        <v>136</v>
+      </c>
+      <c r="K5" s="17" t="s">
+        <v>159</v>
+      </c>
+      <c r="L5" s="6">
+        <v>2</v>
+      </c>
+      <c r="M5" s="6">
+        <f t="shared" si="2"/>
+        <v>200</v>
+      </c>
+      <c r="N5" s="27">
+        <v>210</v>
+      </c>
+      <c r="O5" s="36" t="str">
+        <f t="shared" ref="O5:O31" si="3">HYPERLINK(AB5, "LCSC")</f>
+        <v>LCSC</v>
+      </c>
+      <c r="P5" s="30" t="s">
+        <v>236</v>
+      </c>
+      <c r="Q5" s="7">
+        <f t="shared" si="0"/>
+        <v>39.627000000000002</v>
+      </c>
+      <c r="R5" s="6"/>
+    </row>
+    <row r="6" spans="1:18" s="37" customFormat="1">
+      <c r="A6" s="35"/>
+      <c r="B6" s="9">
+        <f t="shared" si="1"/>
+        <v>4</v>
+      </c>
+      <c r="C6" s="15" t="s">
+        <v>5</v>
+      </c>
+      <c r="D6" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="E6" s="12" t="s">
+        <v>49</v>
+      </c>
+      <c r="F6" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="G6" s="12" t="s">
+        <v>97</v>
+      </c>
+      <c r="H6" s="12" t="s">
+        <v>119</v>
+      </c>
+      <c r="I6" s="6" t="s">
+        <v>179</v>
+      </c>
+      <c r="J6" s="12" t="s">
+        <v>137</v>
+      </c>
+      <c r="K6" s="18" t="s">
+        <v>157</v>
+      </c>
+      <c r="L6" s="12">
+        <v>1</v>
+      </c>
+      <c r="M6" s="6">
+        <f t="shared" si="2"/>
+        <v>100</v>
+      </c>
+      <c r="N6" s="24">
+        <v>200</v>
+      </c>
+      <c r="O6" s="36" t="str">
+        <f t="shared" si="3"/>
+        <v>LCSC</v>
+      </c>
+      <c r="P6" s="25" t="s">
+        <v>189</v>
+      </c>
+      <c r="Q6" s="13">
+        <f t="shared" si="0"/>
+        <v>0.6</v>
+      </c>
+      <c r="R6" s="12"/>
+    </row>
+    <row r="7" spans="1:18" s="37" customFormat="1" ht="24">
+      <c r="A7" s="35"/>
+      <c r="B7" s="8">
+        <f>ROW(B7) - ROW($B$2)</f>
+        <v>5</v>
+      </c>
+      <c r="C7" s="14" t="s">
+        <v>4</v>
+      </c>
+      <c r="D7" s="6" t="s">
+        <v>20</v>
+      </c>
+      <c r="E7" s="6" t="s">
+        <v>50</v>
+      </c>
+      <c r="F7" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="G7" s="6" t="s">
+        <v>98</v>
+      </c>
+      <c r="H7" s="6" t="s">
+        <v>117</v>
+      </c>
+      <c r="I7" s="6" t="s">
+        <v>179</v>
+      </c>
+      <c r="J7" s="6" t="s">
+        <v>138</v>
+      </c>
+      <c r="K7" s="17" t="s">
+        <v>157</v>
+      </c>
+      <c r="L7" s="6">
+        <v>5</v>
+      </c>
+      <c r="M7" s="6">
+        <f t="shared" si="2"/>
+        <v>500</v>
+      </c>
+      <c r="N7" s="27">
+        <v>600</v>
+      </c>
+      <c r="O7" s="36" t="str">
+        <f t="shared" si="3"/>
+        <v>LCSC</v>
+      </c>
+      <c r="P7" s="30" t="s">
+        <v>190</v>
+      </c>
+      <c r="Q7" s="7">
+        <f t="shared" si="0"/>
+        <v>1.02</v>
+      </c>
+      <c r="R7" s="6"/>
+    </row>
+    <row r="8" spans="1:18" s="37" customFormat="1">
+      <c r="A8" s="35"/>
+      <c r="B8" s="9">
+        <f t="shared" si="1"/>
+        <v>6</v>
+      </c>
+      <c r="C8" s="15" t="s">
+        <v>6</v>
+      </c>
+      <c r="D8" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="E8" s="12" t="s">
+        <v>51</v>
+      </c>
+      <c r="F8" s="12" t="s">
+        <v>76</v>
+      </c>
+      <c r="G8" s="12" t="s">
+        <v>99</v>
+      </c>
+      <c r="H8" s="12" t="s">
+        <v>120</v>
+      </c>
+      <c r="I8" s="6" t="s">
+        <v>179</v>
+      </c>
+      <c r="J8" s="12" t="s">
+        <v>139</v>
+      </c>
+      <c r="K8" s="18" t="s">
+        <v>179</v>
+      </c>
+      <c r="L8" s="12">
+        <v>1</v>
+      </c>
+      <c r="M8" s="6">
+        <f t="shared" si="2"/>
+        <v>100</v>
+      </c>
+      <c r="N8" s="24">
+        <v>110</v>
+      </c>
+      <c r="O8" s="36" t="str">
+        <f t="shared" si="3"/>
+        <v>LCSC</v>
+      </c>
+      <c r="P8" s="25" t="s">
+        <v>237</v>
+      </c>
+      <c r="Q8" s="13">
+        <f t="shared" si="0"/>
+        <v>3.1240000000000001</v>
+      </c>
+      <c r="R8" s="12"/>
+    </row>
+    <row r="9" spans="1:18" s="37" customFormat="1">
+      <c r="A9" s="35"/>
+      <c r="B9" s="8">
+        <f>ROW(B9) - ROW($B$2)</f>
+        <v>7</v>
+      </c>
+      <c r="C9" s="14" t="s">
+        <v>6</v>
+      </c>
+      <c r="D9" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="E9" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="F9" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="G9" s="6" t="s">
+        <v>100</v>
+      </c>
+      <c r="H9" s="6" t="s">
+        <v>121</v>
+      </c>
+      <c r="I9" s="6" t="s">
+        <v>179</v>
+      </c>
+      <c r="J9" s="6" t="s">
+        <v>140</v>
+      </c>
+      <c r="K9" s="18" t="s">
+        <v>179</v>
+      </c>
+      <c r="L9" s="6">
+        <v>2</v>
+      </c>
+      <c r="M9" s="6">
+        <f t="shared" si="2"/>
+        <v>200</v>
+      </c>
+      <c r="N9" s="27">
+        <v>210</v>
+      </c>
+      <c r="O9" s="36" t="str">
+        <f t="shared" si="3"/>
+        <v>LCSC</v>
+      </c>
+      <c r="P9" s="30" t="s">
+        <v>194</v>
+      </c>
+      <c r="Q9" s="7">
+        <f t="shared" si="0"/>
+        <v>6.468</v>
+      </c>
+      <c r="R9" s="6"/>
+    </row>
+    <row r="10" spans="1:18" s="37" customFormat="1" ht="60">
+      <c r="A10" s="35"/>
+      <c r="B10" s="9">
+        <f t="shared" si="1"/>
+        <v>8</v>
+      </c>
+      <c r="C10" s="15" t="s">
+        <v>7</v>
+      </c>
+      <c r="D10" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="E10" s="12" t="s">
+        <v>53</v>
+      </c>
+      <c r="F10" s="12" t="s">
+        <v>178</v>
+      </c>
+      <c r="G10" s="12" t="s">
+        <v>78</v>
+      </c>
+      <c r="H10" s="12" t="s">
+        <v>122</v>
+      </c>
+      <c r="I10" s="6" t="s">
+        <v>179</v>
+      </c>
+      <c r="J10" s="12" t="s">
+        <v>141</v>
+      </c>
+      <c r="K10" s="18" t="s">
+        <v>179</v>
+      </c>
+      <c r="L10" s="12">
+        <v>1</v>
+      </c>
+      <c r="M10" s="6">
+        <f t="shared" si="2"/>
+        <v>100</v>
+      </c>
+      <c r="N10" s="24">
+        <v>105</v>
+      </c>
+      <c r="O10" s="36" t="str">
+        <f t="shared" si="3"/>
+        <v>LCSC</v>
+      </c>
+      <c r="P10" s="25" t="s">
+        <v>238</v>
+      </c>
+      <c r="Q10" s="13">
+        <f t="shared" si="0"/>
+        <v>16.506</v>
+      </c>
+      <c r="R10" s="12"/>
+    </row>
+    <row r="11" spans="1:18" s="37" customFormat="1">
+      <c r="A11" s="35"/>
+      <c r="B11" s="8">
+        <f>ROW(B11) - ROW($B$2)</f>
+        <v>9</v>
+      </c>
+      <c r="C11" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="D11" s="6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E11" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="F11" s="12" t="s">
+        <v>178</v>
+      </c>
+      <c r="G11" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="H11" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="I11" s="6" t="s">
+        <v>179</v>
+      </c>
+      <c r="J11" s="6" t="s">
+        <v>179</v>
+      </c>
+      <c r="K11" s="18" t="s">
+        <v>179</v>
+      </c>
+      <c r="L11" s="6">
+        <v>2</v>
+      </c>
+      <c r="M11" s="6">
+        <f t="shared" si="2"/>
+        <v>200</v>
+      </c>
+      <c r="N11" s="27">
+        <v>200</v>
+      </c>
+      <c r="O11" s="36" t="s">
+        <v>208</v>
+      </c>
+      <c r="P11" s="30">
+        <v>0.59399999999999997</v>
+      </c>
+      <c r="Q11" s="7">
+        <f t="shared" si="0"/>
+        <v>118.8</v>
+      </c>
+      <c r="R11" s="6"/>
+    </row>
+    <row r="12" spans="1:18" s="37" customFormat="1" ht="60">
+      <c r="A12" s="35"/>
+      <c r="B12" s="9">
+        <f t="shared" si="1"/>
+        <v>10</v>
+      </c>
+      <c r="C12" s="15" t="s">
+        <v>9</v>
+      </c>
+      <c r="D12" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="E12" s="12" t="s">
+        <v>55</v>
+      </c>
+      <c r="F12" s="12" t="s">
+        <v>80</v>
+      </c>
+      <c r="G12" s="12" t="s">
+        <v>101</v>
+      </c>
+      <c r="H12" s="12" t="s">
+        <v>124</v>
+      </c>
+      <c r="I12" s="6" t="s">
+        <v>179</v>
+      </c>
+      <c r="J12" s="12" t="s">
+        <v>142</v>
+      </c>
+      <c r="K12" s="18" t="s">
+        <v>179</v>
+      </c>
+      <c r="L12" s="12">
+        <v>2</v>
+      </c>
+      <c r="M12" s="6">
+        <f t="shared" si="2"/>
+        <v>200</v>
+      </c>
+      <c r="N12" s="24">
+        <v>200</v>
+      </c>
+      <c r="O12" s="36" t="str">
+        <f t="shared" si="3"/>
+        <v>LCSC</v>
+      </c>
+      <c r="P12" s="25" t="s">
+        <v>239</v>
+      </c>
+      <c r="Q12" s="13">
+        <f t="shared" si="0"/>
+        <v>4.88</v>
+      </c>
+      <c r="R12" s="12"/>
+    </row>
+    <row r="13" spans="1:18" s="37" customFormat="1">
+      <c r="A13" s="35"/>
+      <c r="B13" s="8">
+        <f>ROW(B13) - ROW($B$2)</f>
+        <v>11</v>
+      </c>
+      <c r="C13" s="14" t="s">
+        <v>8</v>
+      </c>
+      <c r="D13" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="E13" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="F13" s="12" t="s">
+        <v>178</v>
+      </c>
+      <c r="G13" s="6" t="s">
+        <v>81</v>
+      </c>
+      <c r="H13" s="6" t="s">
+        <v>123</v>
+      </c>
+      <c r="I13" s="6" t="s">
+        <v>179</v>
+      </c>
+      <c r="J13" s="6" t="s">
+        <v>179</v>
+      </c>
+      <c r="K13" s="18" t="s">
+        <v>179</v>
+      </c>
+      <c r="L13" s="6">
+        <v>4</v>
+      </c>
+      <c r="M13" s="6">
+        <f t="shared" si="2"/>
+        <v>400</v>
+      </c>
+      <c r="N13" s="27">
+        <v>400</v>
+      </c>
+      <c r="O13" s="36" t="s">
+        <v>208</v>
+      </c>
+      <c r="P13" s="30">
+        <v>0.29099999999999998</v>
+      </c>
+      <c r="Q13" s="7">
+        <f t="shared" si="0"/>
+        <v>116.39999999999999</v>
+      </c>
+      <c r="R13" s="6"/>
+    </row>
+    <row r="14" spans="1:18" s="37" customFormat="1">
+      <c r="A14" s="35"/>
+      <c r="B14" s="9">
+        <f t="shared" si="1"/>
+        <v>12</v>
+      </c>
+      <c r="C14" s="15" t="s">
+        <v>8</v>
+      </c>
+      <c r="D14" s="12" t="s">
+        <v>27</v>
+      </c>
+      <c r="E14" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="F14" s="12" t="s">
+        <v>178</v>
+      </c>
+      <c r="G14" s="12" t="s">
+        <v>82</v>
+      </c>
+      <c r="H14" s="12" t="s">
+        <v>123</v>
+      </c>
+      <c r="I14" s="6" t="s">
+        <v>179</v>
+      </c>
+      <c r="J14" s="12" t="s">
+        <v>179</v>
+      </c>
+      <c r="K14" s="18" t="s">
+        <v>179</v>
+      </c>
+      <c r="L14" s="12">
+        <v>3</v>
+      </c>
+      <c r="M14" s="6">
+        <f t="shared" si="2"/>
+        <v>300</v>
+      </c>
+      <c r="N14" s="24">
+        <v>300</v>
+      </c>
+      <c r="O14" s="36" t="s">
+        <v>208</v>
+      </c>
+      <c r="P14" s="25">
+        <v>0.75</v>
+      </c>
+      <c r="Q14" s="13">
+        <f t="shared" si="0"/>
+        <v>225</v>
+      </c>
+      <c r="R14" s="12"/>
+    </row>
+    <row r="15" spans="1:18" s="37" customFormat="1" ht="36">
+      <c r="A15" s="35"/>
+      <c r="B15" s="8">
+        <f>ROW(B15) - ROW($B$2)</f>
+        <v>13</v>
+      </c>
+      <c r="C15" s="14" t="s">
+        <v>10</v>
+      </c>
+      <c r="D15" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="E15" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="F15" s="12" t="s">
+        <v>178</v>
+      </c>
+      <c r="G15" s="6" t="s">
+        <v>83</v>
+      </c>
+      <c r="H15" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="I15" s="6" t="s">
+        <v>179</v>
+      </c>
+      <c r="J15" s="6" t="s">
+        <v>143</v>
+      </c>
+      <c r="K15" s="17" t="s">
+        <v>160</v>
+      </c>
+      <c r="L15" s="6">
+        <v>1</v>
+      </c>
+      <c r="M15" s="6">
+        <f t="shared" si="2"/>
+        <v>100</v>
+      </c>
+      <c r="N15" s="27" t="s">
+        <v>184</v>
+      </c>
+      <c r="O15" s="36" t="str">
+        <f t="shared" si="3"/>
+        <v>LCSC</v>
+      </c>
+      <c r="P15" s="30" t="s">
+        <v>240</v>
+      </c>
+      <c r="Q15" s="7">
+        <f t="shared" si="0"/>
+        <v>59.98</v>
+      </c>
+      <c r="R15" s="6"/>
+    </row>
+    <row r="16" spans="1:18" s="37" customFormat="1" ht="24">
+      <c r="A16" s="35"/>
+      <c r="B16" s="9">
+        <f t="shared" si="1"/>
+        <v>14</v>
+      </c>
+      <c r="C16" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="D16" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="E16" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="F16" s="12" t="s">
+        <v>84</v>
+      </c>
+      <c r="G16" s="12" t="s">
+        <v>102</v>
+      </c>
+      <c r="H16" s="12" t="s">
+        <v>126</v>
+      </c>
+      <c r="I16" s="6" t="s">
+        <v>179</v>
+      </c>
+      <c r="J16" s="12" t="s">
+        <v>144</v>
+      </c>
+      <c r="K16" s="18" t="s">
+        <v>179</v>
+      </c>
+      <c r="L16" s="12">
+        <v>3</v>
+      </c>
+      <c r="M16" s="6">
+        <f t="shared" si="2"/>
+        <v>300</v>
+      </c>
+      <c r="N16" s="24" t="s">
+        <v>248</v>
+      </c>
+      <c r="O16" s="36" t="str">
+        <f t="shared" si="3"/>
+        <v>LCSC</v>
+      </c>
+      <c r="P16" s="25" t="s">
+        <v>241</v>
+      </c>
+      <c r="Q16" s="13">
+        <f t="shared" si="0"/>
+        <v>13.23</v>
+      </c>
+      <c r="R16" s="12"/>
+    </row>
+    <row r="17" spans="1:18" s="37" customFormat="1" ht="48">
+      <c r="A17" s="35"/>
+      <c r="B17" s="8">
+        <f>ROW(B17) - ROW($B$2)</f>
+        <v>15</v>
+      </c>
+      <c r="C17" s="14" t="s">
+        <v>12</v>
+      </c>
+      <c r="D17" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="E17" s="6" t="s">
+        <v>58</v>
+      </c>
+      <c r="F17" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="G17" s="6" t="s">
+        <v>103</v>
+      </c>
+      <c r="H17" s="6" t="s">
+        <v>117</v>
+      </c>
+      <c r="I17" s="6" t="s">
+        <v>179</v>
+      </c>
+      <c r="J17" s="6" t="s">
+        <v>145</v>
+      </c>
+      <c r="K17" s="17" t="s">
+        <v>161</v>
+      </c>
+      <c r="L17" s="6">
+        <v>13</v>
+      </c>
+      <c r="M17" s="6">
+        <f t="shared" si="2"/>
+        <v>1300</v>
+      </c>
+      <c r="N17" s="27" t="s">
+        <v>249</v>
+      </c>
+      <c r="O17" s="36" t="str">
+        <f t="shared" si="3"/>
+        <v>LCSC</v>
+      </c>
+      <c r="P17" s="30" t="s">
+        <v>242</v>
+      </c>
+      <c r="Q17" s="7">
+        <f t="shared" si="0"/>
+        <v>1.04</v>
+      </c>
+      <c r="R17" s="6"/>
+    </row>
+    <row r="18" spans="1:18" s="37" customFormat="1" ht="30">
+      <c r="A18" s="35"/>
+      <c r="B18" s="9">
+        <f t="shared" si="1"/>
+        <v>16</v>
+      </c>
+      <c r="C18" s="15" t="s">
+        <v>13</v>
+      </c>
+      <c r="D18" s="19" t="s">
+        <v>31</v>
+      </c>
+      <c r="E18" s="19" t="s">
+        <v>59</v>
+      </c>
+      <c r="F18" s="19" t="s">
+        <v>86</v>
+      </c>
+      <c r="G18" s="19" t="s">
+        <v>104</v>
+      </c>
+      <c r="H18" s="19" t="s">
+        <v>117</v>
+      </c>
+      <c r="I18" s="6" t="s">
+        <v>179</v>
+      </c>
+      <c r="J18" s="19" t="s">
+        <v>180</v>
+      </c>
+      <c r="K18" s="20" t="s">
+        <v>162</v>
+      </c>
+      <c r="L18" s="19">
+        <v>1</v>
+      </c>
+      <c r="M18" s="6">
+        <f t="shared" si="2"/>
+        <v>100</v>
+      </c>
+      <c r="N18" s="28" t="s">
+        <v>184</v>
+      </c>
+      <c r="O18" s="36" t="str">
+        <f t="shared" si="3"/>
+        <v>LCSC</v>
+      </c>
+      <c r="P18" s="31" t="s">
+        <v>179</v>
+      </c>
+      <c r="Q18" s="21" t="s">
+        <v>179</v>
+      </c>
+      <c r="R18" s="22" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="19" spans="1:18" s="37" customFormat="1">
+      <c r="A19" s="35"/>
+      <c r="B19" s="8">
+        <f>ROW(B19) - ROW($B$2)</f>
+        <v>17</v>
+      </c>
+      <c r="C19" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="D19" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="E19" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="F19" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="G19" s="6" t="s">
+        <v>104</v>
+      </c>
+      <c r="H19" s="6" t="s">
+        <v>117</v>
+      </c>
+      <c r="I19" s="6" t="s">
+        <v>179</v>
+      </c>
+      <c r="J19" s="6" t="s">
+        <v>180</v>
+      </c>
+      <c r="K19" s="17" t="s">
+        <v>161</v>
+      </c>
+      <c r="L19" s="6">
+        <v>1</v>
+      </c>
+      <c r="M19" s="6">
+        <f t="shared" si="2"/>
+        <v>100</v>
+      </c>
+      <c r="N19" s="27" t="s">
+        <v>184</v>
+      </c>
+      <c r="O19" s="36" t="str">
+        <f t="shared" si="3"/>
+        <v>LCSC</v>
+      </c>
+      <c r="P19" s="30" t="s">
+        <v>198</v>
+      </c>
+      <c r="Q19" s="7">
+        <f>P19*N19</f>
+        <v>0.31</v>
+      </c>
+      <c r="R19" s="6"/>
+    </row>
+    <row r="20" spans="1:18" s="37" customFormat="1" ht="24">
+      <c r="A20" s="35"/>
+      <c r="B20" s="9">
+        <f t="shared" si="1"/>
+        <v>18</v>
+      </c>
+      <c r="C20" s="15" t="s">
+        <v>12</v>
+      </c>
+      <c r="D20" s="12" t="s">
+        <v>33</v>
+      </c>
+      <c r="E20" s="12" t="s">
+        <v>60</v>
+      </c>
+      <c r="F20" s="12" t="s">
+        <v>87</v>
+      </c>
+      <c r="G20" s="12" t="s">
+        <v>105</v>
+      </c>
+      <c r="H20" s="12" t="s">
+        <v>117</v>
+      </c>
+      <c r="I20" s="6" t="s">
+        <v>179</v>
+      </c>
+      <c r="J20" s="12" t="s">
+        <v>146</v>
+      </c>
+      <c r="K20" s="18" t="s">
+        <v>163</v>
+      </c>
+      <c r="L20" s="12">
+        <v>4</v>
+      </c>
+      <c r="M20" s="6">
+        <f t="shared" si="2"/>
+        <v>400</v>
+      </c>
+      <c r="N20" s="24" t="s">
+        <v>250</v>
+      </c>
+      <c r="O20" s="36" t="str">
+        <f t="shared" si="3"/>
+        <v>LCSC</v>
+      </c>
+      <c r="P20" s="25" t="s">
+        <v>199</v>
+      </c>
+      <c r="Q20" s="13">
+        <f>P20*N20</f>
+        <v>0.24</v>
+      </c>
+      <c r="R20" s="12"/>
+    </row>
+    <row r="21" spans="1:18" s="37" customFormat="1" ht="24">
+      <c r="A21" s="35"/>
+      <c r="B21" s="8">
+        <f>ROW(B21) - ROW($B$2)</f>
+        <v>19</v>
+      </c>
+      <c r="C21" s="14" t="s">
+        <v>13</v>
+      </c>
+      <c r="D21" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="E21" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="F21" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="G21" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="H21" s="6" t="s">
+        <v>117</v>
+      </c>
+      <c r="I21" s="6" t="s">
+        <v>179</v>
+      </c>
+      <c r="J21" s="6" t="s">
+        <v>147</v>
+      </c>
+      <c r="K21" s="17" t="s">
+        <v>161</v>
+      </c>
+      <c r="L21" s="6">
+        <v>4</v>
+      </c>
+      <c r="M21" s="6">
+        <f t="shared" si="2"/>
+        <v>400</v>
+      </c>
+      <c r="N21" s="27" t="s">
+        <v>250</v>
+      </c>
+      <c r="O21" s="36" t="str">
+        <f t="shared" si="3"/>
+        <v>LCSC</v>
+      </c>
+      <c r="P21" s="30" t="s">
+        <v>199</v>
+      </c>
+      <c r="Q21" s="7">
+        <f>P21*N21</f>
+        <v>0.24</v>
+      </c>
+      <c r="R21" s="6"/>
+    </row>
+    <row r="22" spans="1:18" s="37" customFormat="1">
+      <c r="A22" s="35"/>
+      <c r="B22" s="9">
+        <f t="shared" si="1"/>
+        <v>20</v>
+      </c>
+      <c r="C22" s="15" t="s">
+        <v>12</v>
+      </c>
+      <c r="D22" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="E22" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="F22" s="12" t="s">
+        <v>85</v>
+      </c>
+      <c r="G22" s="12" t="s">
+        <v>107</v>
+      </c>
+      <c r="H22" s="12" t="s">
+        <v>117</v>
+      </c>
+      <c r="I22" s="6" t="s">
+        <v>179</v>
+      </c>
+      <c r="J22" s="12" t="s">
+        <v>148</v>
+      </c>
+      <c r="K22" s="18" t="s">
+        <v>164</v>
+      </c>
+      <c r="L22" s="12">
+        <v>2</v>
+      </c>
+      <c r="M22" s="6">
+        <f t="shared" si="2"/>
+        <v>200</v>
+      </c>
+      <c r="N22" s="24" t="s">
+        <v>251</v>
+      </c>
+      <c r="O22" s="36" t="str">
+        <f t="shared" si="3"/>
+        <v>LCSC</v>
+      </c>
+      <c r="P22" s="25" t="s">
+        <v>200</v>
+      </c>
+      <c r="Q22" s="13">
+        <f>P22*N22</f>
+        <v>0.24</v>
+      </c>
+      <c r="R22" s="12"/>
+    </row>
+    <row r="23" spans="1:18" s="37" customFormat="1" ht="30">
+      <c r="A23" s="35"/>
+      <c r="B23" s="8">
+        <f>ROW(B23) - ROW($B$2)</f>
+        <v>21</v>
+      </c>
+      <c r="C23" s="14" t="s">
+        <v>12</v>
+      </c>
+      <c r="D23" s="19" t="s">
+        <v>36</v>
+      </c>
+      <c r="E23" s="19" t="s">
+        <v>60</v>
+      </c>
+      <c r="F23" s="19" t="s">
+        <v>87</v>
+      </c>
+      <c r="G23" s="19" t="s">
+        <v>105</v>
+      </c>
+      <c r="H23" s="19" t="s">
+        <v>117</v>
+      </c>
+      <c r="I23" s="6" t="s">
+        <v>179</v>
+      </c>
+      <c r="J23" s="19" t="s">
+        <v>146</v>
+      </c>
+      <c r="K23" s="20" t="s">
+        <v>162</v>
+      </c>
+      <c r="L23" s="19">
+        <v>2</v>
+      </c>
+      <c r="M23" s="6">
+        <f t="shared" si="2"/>
+        <v>200</v>
+      </c>
+      <c r="N23" s="28" t="s">
+        <v>251</v>
+      </c>
+      <c r="O23" s="36" t="str">
+        <f t="shared" si="3"/>
+        <v>LCSC</v>
+      </c>
+      <c r="P23" s="31" t="s">
+        <v>179</v>
+      </c>
+      <c r="Q23" s="21" t="s">
+        <v>179</v>
+      </c>
+      <c r="R23" s="22" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="24" spans="1:18" s="37" customFormat="1">
+      <c r="A24" s="35"/>
+      <c r="B24" s="9">
+        <f t="shared" si="1"/>
+        <v>22</v>
+      </c>
+      <c r="C24" s="14" t="s">
+        <v>12</v>
+      </c>
+      <c r="D24" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="E24" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="F24" s="12" t="s">
+        <v>88</v>
+      </c>
+      <c r="G24" s="12" t="s">
+        <v>108</v>
+      </c>
+      <c r="H24" s="12" t="s">
+        <v>127</v>
+      </c>
+      <c r="I24" s="6" t="s">
+        <v>179</v>
+      </c>
+      <c r="J24" s="12" t="s">
+        <v>149</v>
+      </c>
+      <c r="K24" s="18" t="s">
+        <v>165</v>
+      </c>
+      <c r="L24" s="12">
+        <v>3</v>
+      </c>
+      <c r="M24" s="6">
+        <f t="shared" si="2"/>
+        <v>300</v>
+      </c>
+      <c r="N24" s="24" t="s">
+        <v>248</v>
+      </c>
+      <c r="O24" s="36" t="str">
+        <f t="shared" si="3"/>
+        <v>LCSC</v>
+      </c>
+      <c r="P24" s="25" t="s">
+        <v>243</v>
+      </c>
+      <c r="Q24" s="13">
+        <f t="shared" ref="Q24:Q31" si="4">P24*N24</f>
+        <v>11.309999999999999</v>
+      </c>
+      <c r="R24" s="12"/>
+    </row>
+    <row r="25" spans="1:18" s="37" customFormat="1">
+      <c r="A25" s="35"/>
+      <c r="B25" s="8">
+        <f>ROW(B25) - ROW($B$2)</f>
+        <v>23</v>
+      </c>
+      <c r="C25" s="14" t="s">
+        <v>12</v>
+      </c>
+      <c r="D25" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="E25" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="F25" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="G25" s="6" t="s">
+        <v>109</v>
+      </c>
+      <c r="H25" s="6" t="s">
+        <v>117</v>
+      </c>
+      <c r="I25" s="6" t="s">
+        <v>179</v>
+      </c>
+      <c r="J25" s="6" t="s">
+        <v>150</v>
+      </c>
+      <c r="K25" s="17" t="s">
+        <v>166</v>
+      </c>
+      <c r="L25" s="6">
+        <v>3</v>
+      </c>
+      <c r="M25" s="6">
+        <f t="shared" si="2"/>
+        <v>300</v>
+      </c>
+      <c r="N25" s="27" t="s">
+        <v>248</v>
+      </c>
+      <c r="O25" s="36" t="str">
+        <f t="shared" si="3"/>
+        <v>LCSC</v>
+      </c>
+      <c r="P25" s="30" t="s">
+        <v>199</v>
+      </c>
+      <c r="Q25" s="7">
+        <f t="shared" si="4"/>
+        <v>0.18</v>
+      </c>
+      <c r="R25" s="6"/>
+    </row>
+    <row r="26" spans="1:18" s="37" customFormat="1">
+      <c r="A26" s="35"/>
+      <c r="B26" s="9">
+        <f t="shared" si="1"/>
+        <v>24</v>
+      </c>
+      <c r="C26" s="15" t="s">
+        <v>12</v>
+      </c>
+      <c r="D26" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="E26" s="12" t="s">
+        <v>65</v>
+      </c>
+      <c r="F26" s="12" t="s">
+        <v>85</v>
+      </c>
+      <c r="G26" s="12" t="s">
+        <v>110</v>
+      </c>
+      <c r="H26" s="12" t="s">
+        <v>117</v>
+      </c>
+      <c r="I26" s="6" t="s">
+        <v>179</v>
+      </c>
+      <c r="J26" s="12" t="s">
+        <v>151</v>
+      </c>
+      <c r="K26" s="18" t="s">
+        <v>167</v>
+      </c>
+      <c r="L26" s="12">
+        <v>3</v>
+      </c>
+      <c r="M26" s="6">
+        <f t="shared" si="2"/>
+        <v>300</v>
+      </c>
+      <c r="N26" s="24" t="s">
+        <v>248</v>
+      </c>
+      <c r="O26" s="36" t="str">
+        <f t="shared" si="3"/>
+        <v>LCSC</v>
+      </c>
+      <c r="P26" s="25" t="s">
+        <v>200</v>
+      </c>
+      <c r="Q26" s="13">
+        <f t="shared" si="4"/>
+        <v>0.36</v>
+      </c>
+      <c r="R26" s="12"/>
+    </row>
+    <row r="27" spans="1:18" s="37" customFormat="1">
+      <c r="A27" s="35"/>
+      <c r="B27" s="8">
+        <f>ROW(B27) - ROW($B$2)</f>
+        <v>25</v>
+      </c>
+      <c r="C27" s="14" t="s">
+        <v>12</v>
+      </c>
+      <c r="D27" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="E27" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="F27" s="6" t="s">
+        <v>85</v>
+      </c>
+      <c r="G27" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="H27" s="6" t="s">
+        <v>128</v>
+      </c>
+      <c r="I27" s="6" t="s">
+        <v>179</v>
+      </c>
+      <c r="J27" s="6" t="s">
+        <v>152</v>
+      </c>
+      <c r="K27" s="17" t="s">
+        <v>168</v>
+      </c>
+      <c r="L27" s="6">
+        <v>3</v>
+      </c>
+      <c r="M27" s="6">
+        <f t="shared" si="2"/>
+        <v>300</v>
+      </c>
+      <c r="N27" s="27" t="s">
+        <v>248</v>
+      </c>
+      <c r="O27" s="36" t="str">
+        <f t="shared" si="3"/>
+        <v>LCSC</v>
+      </c>
+      <c r="P27" s="30" t="s">
+        <v>200</v>
+      </c>
+      <c r="Q27" s="7">
+        <f t="shared" si="4"/>
+        <v>0.36</v>
+      </c>
+      <c r="R27" s="6"/>
+    </row>
+    <row r="28" spans="1:18" s="37" customFormat="1">
+      <c r="A28" s="35"/>
+      <c r="B28" s="9">
+        <f t="shared" si="1"/>
+        <v>26</v>
+      </c>
+      <c r="C28" s="15" t="s">
+        <v>14</v>
+      </c>
+      <c r="D28" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="E28" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="F28" s="12" t="s">
+        <v>89</v>
+      </c>
+      <c r="G28" s="12" t="s">
+        <v>112</v>
+      </c>
+      <c r="H28" s="12" t="s">
+        <v>129</v>
+      </c>
+      <c r="I28" s="6" t="s">
+        <v>179</v>
+      </c>
+      <c r="J28" s="12" t="s">
+        <v>153</v>
+      </c>
+      <c r="K28" s="18" t="s">
+        <v>179</v>
+      </c>
+      <c r="L28" s="12">
+        <v>1</v>
+      </c>
+      <c r="M28" s="6">
+        <f t="shared" si="2"/>
+        <v>100</v>
+      </c>
+      <c r="N28" s="24" t="s">
+        <v>184</v>
+      </c>
+      <c r="O28" s="36" t="str">
+        <f t="shared" si="3"/>
+        <v>LCSC</v>
+      </c>
+      <c r="P28" s="25" t="s">
+        <v>244</v>
+      </c>
+      <c r="Q28" s="13">
+        <f t="shared" si="4"/>
+        <v>27.67</v>
+      </c>
+      <c r="R28" s="12"/>
+    </row>
+    <row r="29" spans="1:18" s="37" customFormat="1">
+      <c r="A29" s="35"/>
+      <c r="B29" s="8">
+        <f>ROW(B29) - ROW($B$2)</f>
+        <v>27</v>
+      </c>
+      <c r="C29" s="14" t="s">
+        <v>14</v>
+      </c>
+      <c r="D29" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="E29" s="6" t="s">
+        <v>68</v>
+      </c>
+      <c r="F29" s="6" t="s">
+        <v>90</v>
+      </c>
+      <c r="G29" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="H29" s="6" t="s">
+        <v>130</v>
+      </c>
+      <c r="I29" s="6" t="s">
+        <v>179</v>
+      </c>
+      <c r="J29" s="6" t="s">
+        <v>154</v>
+      </c>
+      <c r="K29" s="18" t="s">
+        <v>179</v>
+      </c>
+      <c r="L29" s="6">
+        <v>2</v>
+      </c>
+      <c r="M29" s="6">
+        <f t="shared" si="2"/>
+        <v>200</v>
+      </c>
+      <c r="N29" s="27" t="s">
+        <v>251</v>
+      </c>
+      <c r="O29" s="36" t="str">
+        <f t="shared" si="3"/>
+        <v>LCSC</v>
+      </c>
+      <c r="P29" s="30" t="s">
+        <v>245</v>
+      </c>
+      <c r="Q29" s="7">
+        <f t="shared" si="4"/>
+        <v>34.06</v>
+      </c>
+      <c r="R29" s="6"/>
+    </row>
+    <row r="30" spans="1:18" s="37" customFormat="1" ht="36">
+      <c r="A30" s="35"/>
+      <c r="B30" s="9">
+        <f t="shared" si="1"/>
+        <v>28</v>
+      </c>
+      <c r="C30" s="14" t="s">
+        <v>14</v>
+      </c>
+      <c r="D30" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="E30" s="12" t="s">
+        <v>69</v>
+      </c>
+      <c r="F30" s="12" t="s">
+        <v>91</v>
+      </c>
+      <c r="G30" s="12" t="s">
+        <v>114</v>
+      </c>
+      <c r="H30" s="12" t="s">
+        <v>131</v>
+      </c>
+      <c r="I30" s="6" t="s">
+        <v>179</v>
+      </c>
+      <c r="J30" s="12" t="s">
+        <v>155</v>
+      </c>
+      <c r="K30" s="18" t="s">
+        <v>179</v>
+      </c>
+      <c r="L30" s="12">
+        <v>3</v>
+      </c>
+      <c r="M30" s="6">
+        <f t="shared" si="2"/>
+        <v>300</v>
+      </c>
+      <c r="N30" s="24" t="s">
+        <v>248</v>
+      </c>
+      <c r="O30" s="36" t="str">
+        <f t="shared" si="3"/>
+        <v>LCSC</v>
+      </c>
+      <c r="P30" s="25" t="s">
+        <v>246</v>
+      </c>
+      <c r="Q30" s="13">
+        <f t="shared" si="4"/>
+        <v>60.54</v>
+      </c>
+      <c r="R30" s="12"/>
+    </row>
+    <row r="31" spans="1:18" s="37" customFormat="1" ht="24.75" thickBot="1">
+      <c r="A31" s="35"/>
+      <c r="B31" s="8">
+        <f>ROW(B31) - ROW($B$2)</f>
+        <v>29</v>
+      </c>
+      <c r="C31" s="14" t="s">
+        <v>14</v>
+      </c>
+      <c r="D31" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="E31" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="F31" s="6" t="s">
+        <v>92</v>
+      </c>
+      <c r="G31" s="6" t="s">
+        <v>115</v>
+      </c>
+      <c r="H31" s="6" t="s">
+        <v>132</v>
+      </c>
+      <c r="I31" s="6" t="s">
+        <v>179</v>
+      </c>
+      <c r="J31" s="6" t="s">
+        <v>156</v>
+      </c>
+      <c r="K31" s="18" t="s">
+        <v>179</v>
+      </c>
+      <c r="L31" s="6">
+        <v>3</v>
+      </c>
+      <c r="M31" s="6">
+        <f t="shared" si="2"/>
+        <v>300</v>
+      </c>
+      <c r="N31" s="27" t="s">
+        <v>248</v>
+      </c>
+      <c r="O31" s="38" t="str">
+        <f t="shared" si="3"/>
+        <v>LCSC</v>
+      </c>
+      <c r="P31" s="30" t="s">
+        <v>247</v>
+      </c>
+      <c r="Q31" s="7">
+        <f t="shared" si="4"/>
+        <v>41.940000000000005</v>
+      </c>
+      <c r="R31" s="6"/>
+    </row>
+    <row r="32" spans="1:18" ht="19.5" thickBot="1">
+      <c r="A32" s="1"/>
+      <c r="B32" s="1"/>
+      <c r="C32" s="1"/>
+      <c r="D32" s="1"/>
+      <c r="E32" s="1"/>
+      <c r="F32" s="1"/>
+      <c r="G32" s="1"/>
+      <c r="H32" s="1"/>
+      <c r="I32" s="1"/>
+      <c r="J32" s="1"/>
+      <c r="K32" s="1"/>
+      <c r="L32" s="1"/>
+      <c r="M32" s="1"/>
+      <c r="N32" s="40" t="s">
+        <v>1</v>
+      </c>
+      <c r="O32" s="41"/>
+      <c r="P32" s="41"/>
+      <c r="Q32" s="10">
+        <f>SUM(Q3:Q31)</f>
+        <v>801.05699999999979</v>
+      </c>
+      <c r="R32" s="1"/>
+    </row>
+    <row r="33" spans="1:18" ht="19.5" thickBot="1">
+      <c r="A33" s="1"/>
+      <c r="B33" s="1"/>
+      <c r="C33" s="1"/>
+      <c r="D33" s="1"/>
+      <c r="E33" s="1"/>
+      <c r="F33" s="1"/>
+      <c r="G33" s="1"/>
+      <c r="H33" s="1"/>
+      <c r="I33" s="1"/>
+      <c r="J33" s="1"/>
+      <c r="K33" s="1"/>
+      <c r="L33" s="1"/>
+      <c r="M33" s="1"/>
+      <c r="N33" s="40" t="s">
+        <v>2</v>
+      </c>
+      <c r="O33" s="41"/>
+      <c r="P33" s="41"/>
+      <c r="Q33" s="11">
+        <f>Q32/100</f>
+        <v>8.0105699999999977</v>
+      </c>
+      <c r="R33" s="1"/>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="K1:R1"/>
+    <mergeCell ref="N32:P32"/>
+    <mergeCell ref="N33:P33"/>
+  </mergeCells>
+  <hyperlinks>
+    <hyperlink ref="O11" r:id="rId1"/>
+    <hyperlink ref="O13" r:id="rId2"/>
+    <hyperlink ref="O14" r:id="rId3"/>
+    <hyperlink ref="O3" r:id="rId4"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>